<commit_message>
Quota change model added as chapter and to the table
</commit_message>
<xml_diff>
--- a/Index_table.xlsx
+++ b/Index_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samantha.l.werner\Desktop\Github\READ-SSB-SSB_METRICS_CATALOG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCA3E37-4771-43F1-B38C-9C765F6396BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1432FD1-4C12-47F2-A43A-B942E99F0C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22550" yWindow="140" windowWidth="13300" windowHeight="10470" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
+    <workbookView xWindow="19850" yWindow="710" windowWidth="14430" windowHeight="10650" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -96,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="124">
   <si>
     <t xml:space="preserve">Metric Category </t>
   </si>
@@ -484,6 +481,24 @@
   </si>
   <si>
     <t>Vessel-level</t>
+  </si>
+  <si>
+    <t>Sector component of the groundfish fishery</t>
+  </si>
+  <si>
+    <t>Quota Change Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ports and Vessel Length </t>
+  </si>
+  <si>
+    <t>2020- Most Recent Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Revenue</t>
+  </si>
+  <si>
+    <t>Opperating Profit</t>
   </si>
 </sst>
 </file>
@@ -677,7 +692,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -700,19 +715,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -753,9 +759,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -793,7 +799,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -899,7 +905,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1041,7 +1047,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1049,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D40A82-FAB7-4053-BBD9-44EE0830FAC1}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="20.3828125" customWidth="1"/>
@@ -1088,22 +1094,22 @@
       <c r="A2" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1126,7 +1132,7 @@
       <c r="F3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1149,7 +1155,7 @@
       <c r="F4" s="4">
         <v>2022</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1172,7 +1178,7 @@
       <c r="F5" s="4">
         <v>2022</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1195,7 +1201,7 @@
       <c r="F6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1218,7 +1224,7 @@
       <c r="F7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1238,10 +1244,10 @@
       <c r="E8" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="5" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1261,10 +1267,10 @@
       <c r="E9" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="5" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1284,10 +1290,10 @@
       <c r="E10" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="5" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1307,10 +1313,10 @@
       <c r="E11" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="5" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1330,10 +1336,10 @@
       <c r="E12" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="5" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1353,79 +1359,79 @@
       <c r="E13" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G14" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F15" s="4">
-        <v>2024</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F16" s="4">
-        <v>2024</v>
-      </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1434,7 +1440,7 @@
         <v>104</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>108</v>
@@ -1448,7 +1454,7 @@
       <c r="F17" s="4">
         <v>2024</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1457,7 +1463,7 @@
         <v>104</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>108</v>
@@ -1471,145 +1477,145 @@
       <c r="F18" s="4">
         <v>2024</v>
       </c>
-      <c r="G18" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="51.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="5" t="s">
+      <c r="G18" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="4">
+        <v>2024</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F20" s="4">
+        <v>2024</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="51.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B21" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="28.3" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="5" t="s">
+      <c r="G21" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="28.3" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B22" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F22" s="5">
         <v>2022</v>
       </c>
-      <c r="G20" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="9" t="s">
+      <c r="G22" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B23" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C23" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D23" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E23" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F23" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G21" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="55.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="9" t="s">
+      <c r="G23" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="55.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B24" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C24" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="5" t="s">
         <v>117</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1617,22 +1623,22 @@
       <c r="A25" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="B25" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G25" s="9" t="s">
+      <c r="E25" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G25" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1641,21 +1647,21 @@
         <v>21</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="9" t="s">
-        <v>35</v>
+      <c r="E26" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="G26" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1664,12 +1670,12 @@
         <v>21</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="5" t="s">
         <v>117</v>
       </c>
       <c r="E27" s="4" t="s">
@@ -1678,191 +1684,191 @@
       <c r="F27" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G27" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G27" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A28" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G28" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G28" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A29" s="7" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>111</v>
+        <v>29</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>116</v>
+        <v>6</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A30" s="7" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>116</v>
+        <v>6</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="77.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A31" s="7" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>113</v>
+        <v>30</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+        <v>119</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A32" s="7" t="s">
         <v>110</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="5" t="s">
         <v>116</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G32" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G32" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A33" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>43</v>
+        <v>112</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>63</v>
+        <v>115</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+        <v>18</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A34" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>44</v>
+        <v>113</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>63</v>
+        <v>115</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+        <v>18</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A35" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>45</v>
+        <v>114</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>63</v>
+        <v>115</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G35" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G35" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1871,7 +1877,7 @@
         <v>60</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>61</v>
@@ -1879,22 +1885,22 @@
       <c r="D36" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G36" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G36" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>61</v>
@@ -1902,13 +1908,13 @@
       <c r="D37" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1917,7 +1923,7 @@
         <v>60</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>61</v>
@@ -1925,13 +1931,13 @@
       <c r="D38" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="E38" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="G38" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1940,7 +1946,7 @@
         <v>60</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>61</v>
@@ -1948,13 +1954,13 @@
       <c r="D39" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="G39" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1963,7 +1969,7 @@
         <v>60</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>61</v>
@@ -1971,13 +1977,13 @@
       <c r="D40" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="G40" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1986,7 +1992,7 @@
         <v>60</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>61</v>
@@ -1994,13 +2000,13 @@
       <c r="D41" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G41" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2009,7 +2015,7 @@
         <v>60</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>61</v>
@@ -2017,13 +2023,13 @@
       <c r="D42" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E42" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G42" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2032,7 +2038,7 @@
         <v>60</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>61</v>
@@ -2040,13 +2046,13 @@
       <c r="D43" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G43" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2055,7 +2061,7 @@
         <v>60</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>61</v>
@@ -2063,22 +2069,22 @@
       <c r="D44" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E44" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G44" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G44" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A45" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>61</v>
@@ -2086,13 +2092,13 @@
       <c r="D45" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2101,274 +2107,343 @@
         <v>60</v>
       </c>
       <c r="B46" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A48" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A49" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C46" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B47" s="4" t="s">
+      <c r="C49" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A50" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C47" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A48" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B48" s="4" t="s">
+      <c r="C50" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A51" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C48" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A49" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B49" s="4" t="s">
+      <c r="C51" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A52" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B50" s="4" t="s">
+      <c r="C52" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A53" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C50" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A51" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B51" s="4" t="s">
+      <c r="C53" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A54" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C51" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F51" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A52" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B52" s="4" t="s">
+      <c r="C54" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A55" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C52" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A53" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B53" s="4" t="s">
+      <c r="C55" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A56" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A54" s="10" t="s">
+      <c r="C56" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A57" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C57" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="D57" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E54" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="F54" s="9" t="s">
+      <c r="E57" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F57" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G54" s="12" t="s">
+      <c r="G57" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A55" s="10" t="s">
+    <row r="58" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A58" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B58" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C58" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="D58" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E55" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F55" s="9" t="s">
+      <c r="E58" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F58" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="G58" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A56" s="10" t="s">
+    <row r="59" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A59" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B56" s="9" t="s">
+      <c r="B59" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C59" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D56" s="9" t="s">
+      <c r="D59" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E56" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F56" s="9" t="s">
+      <c r="E59" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F59" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="G59" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="28.3" x14ac:dyDescent="0.4">
-      <c r="A57" s="10" t="s">
+    <row r="60" spans="1:7" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A60" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="9" t="s">
+      <c r="B60" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C60" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D57" s="9" t="s">
+      <c r="D60" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E57" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F57" s="9" t="s">
+      <c r="E60" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F60" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G60" s="5" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2424,25 +2499,25 @@
       <c r="A2" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2468,7 +2543,7 @@
       <c r="G3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2494,7 +2569,7 @@
       <c r="G4" s="4">
         <v>2022</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2520,7 +2595,7 @@
       <c r="G5" s="4">
         <v>2022</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2546,7 +2621,7 @@
       <c r="G6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2572,7 +2647,7 @@
       <c r="G7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2583,7 +2658,7 @@
       <c r="B8" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>67</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -2595,10 +2670,10 @@
       <c r="F8" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="5" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2609,7 +2684,7 @@
       <c r="B9" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="10" t="s">
         <v>68</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -2621,10 +2696,10 @@
       <c r="F9" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="5" t="s">
         <v>94</v>
       </c>
     </row>
@@ -2635,7 +2710,7 @@
       <c r="B10" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>69</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -2647,10 +2722,10 @@
       <c r="F10" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="5" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2661,7 +2736,7 @@
       <c r="B11" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>70</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -2673,10 +2748,10 @@
       <c r="F11" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="5" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2687,7 +2762,7 @@
       <c r="B12" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="10" t="s">
         <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -2699,10 +2774,10 @@
       <c r="F12" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="5" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2713,7 +2788,7 @@
       <c r="B13" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="10" t="s">
         <v>72</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -2725,10 +2800,10 @@
       <c r="F13" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2737,21 +2812,21 @@
         <v>97</v>
       </c>
       <c r="B14" s="4"/>
-      <c r="C14" s="14"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="9"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="5" t="s">
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D15" s="6" t="s">
@@ -2766,21 +2841,21 @@
       <c r="G15" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="4" t="s">
@@ -2789,62 +2864,62 @@
       <c r="F16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="5">
         <v>2022</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15.45" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="C17" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="C18" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>6</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2855,13 +2930,13 @@
       <c r="B19" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F19" s="6" t="s">
@@ -2870,7 +2945,7 @@
       <c r="G19" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2881,7 +2956,7 @@
       <c r="B20" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D20" s="4" t="s">
@@ -2896,7 +2971,7 @@
       <c r="G20" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2907,7 +2982,7 @@
       <c r="B21" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D21" s="4" t="s">
@@ -2922,7 +2997,7 @@
       <c r="G21" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2933,13 +3008,13 @@
       <c r="B22" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F22" s="4" t="s">
@@ -2948,7 +3023,7 @@
       <c r="G22" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2959,7 +3034,7 @@
       <c r="B23" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D23" s="4" t="s">
@@ -2974,7 +3049,7 @@
       <c r="G23" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2985,13 +3060,13 @@
       <c r="B24" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F24" s="4" t="s">
@@ -3000,7 +3075,7 @@
       <c r="G24" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="H24" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3011,13 +3086,13 @@
       <c r="B25" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F25" s="4" t="s">
@@ -3026,7 +3101,7 @@
       <c r="G25" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3037,13 +3112,13 @@
       <c r="B26" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F26" s="4" t="s">
@@ -3052,7 +3127,7 @@
       <c r="G26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3063,13 +3138,13 @@
       <c r="B27" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F27" s="4" t="s">
@@ -3078,7 +3153,7 @@
       <c r="G27" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3089,13 +3164,13 @@
       <c r="B28" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F28" s="4" t="s">
@@ -3104,7 +3179,7 @@
       <c r="G28" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="H28" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3115,13 +3190,13 @@
       <c r="B29" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C29" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F29" s="4" t="s">
@@ -3130,7 +3205,7 @@
       <c r="G29" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="H29" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3141,13 +3216,13 @@
       <c r="B30" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C30" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F30" s="4" t="s">
@@ -3156,7 +3231,7 @@
       <c r="G30" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3167,13 +3242,13 @@
       <c r="B31" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="C31" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F31" s="4" t="s">
@@ -3182,7 +3257,7 @@
       <c r="G31" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="H31" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3193,13 +3268,13 @@
       <c r="B32" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F32" s="4" t="s">
@@ -3208,7 +3283,7 @@
       <c r="G32" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H32" s="9" t="s">
+      <c r="H32" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3219,13 +3294,13 @@
       <c r="B33" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="C33" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F33" s="4" t="s">
@@ -3234,7 +3309,7 @@
       <c r="G33" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="H33" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3245,13 +3320,13 @@
       <c r="B34" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C34" s="14" t="s">
+      <c r="C34" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="E34" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F34" s="4" t="s">
@@ -3260,7 +3335,7 @@
       <c r="G34" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3271,13 +3346,13 @@
       <c r="B35" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C35" s="14" t="s">
+      <c r="C35" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F35" s="4" t="s">
@@ -3286,7 +3361,7 @@
       <c r="G35" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="H35" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3297,13 +3372,13 @@
       <c r="B36" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="14" t="s">
+      <c r="C36" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F36" s="4" t="s">
@@ -3312,7 +3387,7 @@
       <c r="G36" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H36" s="9" t="s">
+      <c r="H36" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3323,13 +3398,13 @@
       <c r="B37" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="14" t="s">
+      <c r="C37" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F37" s="4" t="s">
@@ -3338,7 +3413,7 @@
       <c r="G37" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3349,13 +3424,13 @@
       <c r="B38" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="14" t="s">
+      <c r="C38" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="E38" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F38" s="4" t="s">
@@ -3364,7 +3439,7 @@
       <c r="G38" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="H38" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3375,13 +3450,13 @@
       <c r="B39" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="C39" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F39" s="4" t="s">
@@ -3390,7 +3465,7 @@
       <c r="G39" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="H39" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3401,13 +3476,13 @@
       <c r="B40" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="C40" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F40" s="4" t="s">
@@ -3416,7 +3491,7 @@
       <c r="G40" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="H40" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3427,13 +3502,13 @@
       <c r="B41" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="C41" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E41" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F41" s="4" t="s">
@@ -3442,24 +3517,24 @@
       <c r="G41" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H41" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H41" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="71.150000000000006" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A42" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="C42" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E42" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F42" s="4" t="s">
@@ -3468,7 +3543,7 @@
       <c r="G42" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H42" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3479,13 +3554,13 @@
       <c r="B43" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C43" s="14" t="s">
+      <c r="C43" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F43" s="4" t="s">
@@ -3494,7 +3569,7 @@
       <c r="G43" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="H43" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3505,13 +3580,13 @@
       <c r="B44" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C44" s="14" t="s">
+      <c r="C44" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E44" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F44" s="4" t="s">
@@ -3520,7 +3595,7 @@
       <c r="G44" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="5" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3531,13 +3606,13 @@
       <c r="B45" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="14" t="s">
+      <c r="C45" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F45" s="4" t="s">
@@ -3546,18 +3621,18 @@
       <c r="G45" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="30.45" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="10" t="s">
+      <c r="A46" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C46" s="13" t="s">
+      <c r="C46" s="10" t="s">
         <v>66</v>
       </c>
       <c r="D46" s="4" t="s">
@@ -3569,88 +3644,88 @@
       <c r="F46" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G46" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H46" s="12" t="s">
+      <c r="H46" s="9" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="57" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D47" s="9" t="s">
+      <c r="D47" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E47" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F47" s="9" t="s">
+      <c r="E47" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F47" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="H47" s="5" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A48" s="10" t="s">
+      <c r="A48" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="B48" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D48" s="9" t="s">
+      <c r="D48" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E48" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F48" s="9" t="s">
+      <c r="E48" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F48" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H48" s="9" t="s">
+      <c r="H48" s="5" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="28.3" x14ac:dyDescent="0.4">
-      <c r="A49" s="10" t="s">
+      <c r="A49" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B49" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E49" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F49" s="9" t="s">
+      <c r="E49" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F49" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G49" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H49" s="9" t="s">
+      <c r="H49" s="5" t="s">
         <v>87</v>
       </c>
     </row>

</xml_diff>